<commit_message>
EmailTextToPay UI Verification Test Cases
</commit_message>
<xml_diff>
--- a/KatalonData/Bootstrap/VT-Data.xlsx
+++ b/KatalonData/Bootstrap/VT-Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t465179\Documents\git\VPS-Katalon\VPS-Katalon\KatalonData\Bootstrap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CAE89DD-B7AF-43D4-92A8-0D1A1BA01BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{340F8E24-4C89-49E1-A404-2A2EBF73FDC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" tabRatio="771" firstSheet="19" activeTab="24" xr2:uid="{F6D5B6E5-5530-44B1-A3FD-270D512FE765}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" tabRatio="771" firstSheet="12" activeTab="17" xr2:uid="{F6D5B6E5-5530-44B1-A3FD-270D512FE765}"/>
   </bookViews>
   <sheets>
     <sheet name="VT-AuthCapVoid-Generic" sheetId="25" r:id="rId1"/>

</xml_diff>

<commit_message>
Added Test Data and Object Repository for Dual CF CF is Creditable
</commit_message>
<xml_diff>
--- a/KatalonData/Bootstrap/VT-Data.xlsx
+++ b/KatalonData/Bootstrap/VT-Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t465179\Documents\git\VPS-Katalon\VPS-Katalon\KatalonData\Bootstrap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{340F8E24-4C89-49E1-A404-2A2EBF73FDC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13705B27-92A9-490F-8731-0F4D7DDA9210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" tabRatio="771" firstSheet="12" activeTab="17" xr2:uid="{F6D5B6E5-5530-44B1-A3FD-270D512FE765}"/>
+    <workbookView xWindow="45972" yWindow="2952" windowWidth="30936" windowHeight="16776" tabRatio="771" firstSheet="13" activeTab="18" xr2:uid="{F6D5B6E5-5530-44B1-A3FD-270D512FE765}"/>
   </bookViews>
   <sheets>
     <sheet name="VT-AuthCapVoid-Generic" sheetId="25" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6278" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6330" uniqueCount="114">
   <si>
     <t>Result</t>
   </si>
@@ -395,6 +395,12 @@
   </si>
   <si>
     <t>2029</t>
+  </si>
+  <si>
+    <t>1032</t>
+  </si>
+  <si>
+    <t>a_Access AutoDualCFtpCFcreditableQA</t>
   </si>
 </sst>
 </file>
@@ -9586,7 +9592,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB20E3F1-C4A0-4DB3-BD74-0C25E6E1CBA8}">
-  <dimension ref="A1:AI9"/>
+  <dimension ref="A1:AI11"/>
   <sheetFormatPr defaultColWidth="12.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="6.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
@@ -9594,7 +9600,7 @@
     <col min="3" max="3" width="6.33203125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="5" max="5" width="9.59765625" style="1" customWidth="1" collapsed="1"/>
-    <col min="6" max="6" width="27.06640625" style="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="35.06640625" style="1" customWidth="1" collapsed="1"/>
     <col min="7" max="7" width="11.59765625" style="1" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="8" max="8" width="32.33203125" style="1" customWidth="1" collapsed="1"/>
     <col min="9" max="9" width="10.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
@@ -10467,6 +10473,166 @@
         <v>57</v>
       </c>
       <c r="AI9" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:35" x14ac:dyDescent="0.45">
+      <c r="D10" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q10" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="S10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="V10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="W10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="X10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AA10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AD10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE10" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG10" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AH10" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AI10" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:35" x14ac:dyDescent="0.45">
+      <c r="D11" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q11" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="S11" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="V11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="W11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="X11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z11" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AA11" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB11" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AD11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG11" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AH11" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AI11" s="1" t="s">
         <v>70</v>
       </c>
     </row>

</xml_diff>